<commit_message>
⏱ All Timeframe scan [2026-09-14]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -3140,7 +3140,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>101786.99 - 115617.15 DR DEMAND</t>
+          <t>101787.0 - 115617.15 DR DEMAND</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -9050,7 +9050,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>10163.49 - 12763.22 DR DEMAND</t>
+          <t>10163.48 - 12763.22 DR DEMAND</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -25850,12 +25850,12 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>52.14 - 68.65 DR DEMAND</t>
+          <t>57.91 - 70.94 DR DEMAND</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>3.0 C</t>
+          <t>4.0 C</t>
         </is>
       </c>
       <c r="J243" t="inlineStr">
@@ -28926,7 +28926,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>1598.44 - 1928.41 RD SUPPLY</t>
+          <t>1598.43 - 1928.41 RD SUPPLY</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -40664,12 +40664,12 @@
       </c>
       <c r="H388" t="inlineStr">
         <is>
-          <t>— NO ACTIVE ZONE —</t>
+          <t>1306.56 - 1466.62 RD SUPPLY</t>
         </is>
       </c>
       <c r="I388" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5.0 C</t>
         </is>
       </c>
       <c r="J388" t="inlineStr">
@@ -40714,7 +40714,7 @@
       </c>
       <c r="R388" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="S388" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-09-15]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -1844,7 +1844,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>101787.0 - 115617.15 DR DEMAND</t>
+          <t>101786.99 - 115617.15 DR DEMAND</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -31186,7 +31186,7 @@
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>1598.44 - 1928.41 RD SUPPLY</t>
+          <t>1598.43 - 1928.41 RD SUPPLY</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
@@ -33532,7 +33532,7 @@
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>4335.0 - 4897.45 RD SUPPLY</t>
+          <t>4334.99 - 4897.45 RD SUPPLY</t>
         </is>
       </c>
       <c r="I318" t="inlineStr">
@@ -38640,7 +38640,7 @@
       </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>550.35 - 680.06 DR DEMAND</t>
+          <t>550.35 - 680.07 DR DEMAND</t>
         </is>
       </c>
       <c r="I368" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-09-16]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -2252,7 +2252,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>101786.99 - 115617.15 DR DEMAND</t>
+          <t>101786.99 - 115617.16 DR DEMAND</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -22450,7 +22450,7 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>4335.0 - 4897.45 RD SUPPLY</t>
+          <t>4334.99 - 4897.45 RD SUPPLY</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-09-17]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -16476,7 +16476,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>10163.48 - 12763.22 DR DEMAND</t>
+          <t>10163.49 - 12763.22 DR DEMAND</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -20856,7 +20856,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1598.43 - 1928.41 RD SUPPLY</t>
+          <t>1598.44 - 1928.41 RD SUPPLY</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -23078,7 +23078,7 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>4335.0 - 4897.45 RD SUPPLY</t>
+          <t>4334.99 - 4897.45 RD SUPPLY</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-09-18]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -14214,7 +14214,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>10163.49 - 12763.22 DR DEMAND</t>
+          <t>10163.48 - 12763.22 DR DEMAND</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -19608,7 +19608,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>4335.0 - 4897.45 RD SUPPLY</t>
+          <t>4334.99 - 4897.45 RD SUPPLY</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-09-21]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -14946,7 +14946,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>10163.48 - 12763.22 DR DEMAND</t>
+          <t>10163.49 - 12763.22 DR DEMAND</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -25332,7 +25332,7 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>101787.0 - 115617.15 DR DEMAND</t>
+          <t>101786.99 - 115617.16 DR DEMAND</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-09-22]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -14616,7 +14616,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>10163.49 - 12763.22 DR DEMAND</t>
+          <t>10163.48 - 12763.22 DR DEMAND</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -20136,7 +20136,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>4334.99 - 4897.45 RD SUPPLY</t>
+          <t>4335.0 - 4897.45 RD SUPPLY</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -21990,7 +21990,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>1598.43 - 1928.41 RD SUPPLY</t>
+          <t>1598.44 - 1928.41 RD SUPPLY</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -22406,7 +22406,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>550.35 - 680.07 DR DEMAND</t>
+          <t>550.35 - 680.06 DR DEMAND</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-09-24]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -27704,7 +27704,7 @@
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>4334.99 - 4897.45 RD SUPPLY</t>
+          <t>4335.0 - 4897.45 RD SUPPLY</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
@@ -39664,7 +39664,7 @@
       </c>
       <c r="H376" t="inlineStr">
         <is>
-          <t>550.35 - 680.07 DR DEMAND</t>
+          <t>550.35 - 680.06 DR DEMAND</t>
         </is>
       </c>
       <c r="I376" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-09-25]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -24288,7 +24288,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>101787.0 - 115617.15 DR DEMAND</t>
+          <t>101786.99 - 115617.15 DR DEMAND</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
@@ -31650,7 +31650,7 @@
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>4335.0 - 4897.45 RD SUPPLY</t>
+          <t>4334.99 - 4897.45 RD SUPPLY</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
@@ -40046,7 +40046,7 @@
       </c>
       <c r="H380" t="inlineStr">
         <is>
-          <t>550.35 - 680.07 DR DEMAND</t>
+          <t>550.35 - 680.06 DR DEMAND</t>
         </is>
       </c>
       <c r="I380" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-09-29]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -22346,7 +22346,7 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>101786.99 - 115617.15 DR DEMAND</t>
+          <t>101787.0 - 115617.15 DR DEMAND</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
@@ -25862,7 +25862,7 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>4334.99 - 4897.45 RD SUPPLY</t>
+          <t>4335.0 - 4897.45 RD SUPPLY</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-09-30]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -29340,7 +29340,7 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>4334.99 - 4897.45 RD SUPPLY</t>
+          <t>4335.0 - 4897.45 RD SUPPLY</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
@@ -31090,7 +31090,7 @@
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>101787.0 - 115617.15 DR DEMAND</t>
+          <t>101786.99 - 115617.16 DR DEMAND</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
@@ -37234,7 +37234,7 @@
       </c>
       <c r="H355" t="inlineStr">
         <is>
-          <t>550.35 - 680.07 DR DEMAND</t>
+          <t>550.35 - 680.06 DR DEMAND</t>
         </is>
       </c>
       <c r="I355" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-10-01]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -20188,7 +20188,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>807.81 - 997.31 DR DEMAND</t>
+          <t>807.83 - 997.32 DR DEMAND</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -29764,7 +29764,7 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>1598.44 - 1928.41 RD SUPPLY</t>
+          <t>1598.43 - 1928.41 RD SUPPLY</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-10-05]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -14592,12 +14592,12 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>52.14 - 68.65 DR DEMAND</t>
+          <t>57.91 - 70.94 DR DEMAND</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>3.0 C</t>
+          <t>4.0 C</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -36198,7 +36198,7 @@
       </c>
       <c r="H345" t="inlineStr">
         <is>
-          <t>550.35 - 680.06 DR DEMAND</t>
+          <t>550.35 - 680.07 DR DEMAND</t>
         </is>
       </c>
       <c r="I345" t="inlineStr">
@@ -38952,12 +38952,12 @@
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>— NO ACTIVE ZONE —</t>
+          <t>633.63 - 764.17 RD SUPPLY</t>
         </is>
       </c>
       <c r="I372" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>4.0 C</t>
         </is>
       </c>
       <c r="J372" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-10-14]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -31188,7 +31188,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>4335.0 - 4897.45 RD SUPPLY</t>
+          <t>4334.99 - 4897.45 RD SUPPLY</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -43968,7 +43968,7 @@
       </c>
       <c r="F419" t="inlineStr">
         <is>
-          <t>6402.71 - 6552.65 RD SUPPLY</t>
+          <t>6402.72 - 6552.65 RD SUPPLY</t>
         </is>
       </c>
       <c r="G419" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-10-15]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -26110,7 +26110,7 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>550.35 - 680.06 DR DEMAND</t>
+          <t>550.35 - 680.07 DR DEMAND</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
@@ -40038,7 +40038,7 @@
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t>6402.72 - 6552.65 RD SUPPLY</t>
+          <t>6402.71 - 6552.65 RD SUPPLY</t>
         </is>
       </c>
       <c r="G380" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-10-16]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -25474,7 +25474,7 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>550.35 - 680.06 DR DEMAND</t>
+          <t>550.35 - 680.07 DR DEMAND</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
@@ -30082,7 +30082,7 @@
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>4334.99 - 4897.45 RD SUPPLY</t>
+          <t>4335.0 - 4897.45 RD SUPPLY</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-10-20]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -27398,7 +27398,7 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>550.35 - 680.07 DR DEMAND</t>
+          <t>550.35 - 680.06 DR DEMAND</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
@@ -35340,7 +35340,7 @@
       </c>
       <c r="H334" t="inlineStr">
         <is>
-          <t>4335.0 - 4897.45 RD SUPPLY</t>
+          <t>4334.99 - 4897.45 RD SUPPLY</t>
         </is>
       </c>
       <c r="I334" t="inlineStr">
@@ -39436,7 +39436,7 @@
       </c>
       <c r="H374" t="inlineStr">
         <is>
-          <t>101786.99 - 115617.15 DR DEMAND</t>
+          <t>101787.0 - 115617.15 DR DEMAND</t>
         </is>
       </c>
       <c r="I374" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-10-21]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -12112,7 +12112,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>4334.99 - 4897.45 RD SUPPLY</t>
+          <t>4335.0 - 4897.45 RD SUPPLY</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -33782,7 +33782,7 @@
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>6402.71 - 6552.65 RD SUPPLY</t>
+          <t>6402.72 - 6552.65 RD SUPPLY</t>
         </is>
       </c>
       <c r="G320" t="inlineStr">
@@ -34710,7 +34710,7 @@
       </c>
       <c r="H329" t="inlineStr">
         <is>
-          <t>101787.0 - 115617.15 DR DEMAND</t>
+          <t>101786.99 - 115617.15 DR DEMAND</t>
         </is>
       </c>
       <c r="I329" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-10-22]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -4172,7 +4172,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>6402.71 - 6552.65 RD SUPPLY</t>
+          <t>6402.72 - 6552.65 RD SUPPLY</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -38268,7 +38268,7 @@
       </c>
       <c r="H365" t="inlineStr">
         <is>
-          <t>550.35 - 680.06 DR DEMAND</t>
+          <t>550.35 - 680.07 DR DEMAND</t>
         </is>
       </c>
       <c r="I365" t="inlineStr">

</xml_diff>

<commit_message>
⏱ All Timeframe scan [2026-10-23]
</commit_message>
<xml_diff>
--- a/NIFTY500_GTF_Dashboard.xlsx
+++ b/NIFTY500_GTF_Dashboard.xlsx
@@ -3108,7 +3108,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>101786.99 - 115617.15 DR DEMAND</t>
+          <t>101787.0 - 115617.15 DR DEMAND</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -35302,7 +35302,7 @@
       </c>
       <c r="H337" t="inlineStr">
         <is>
-          <t>550.35 - 680.07 DR DEMAND</t>
+          <t>550.35 - 680.06 DR DEMAND</t>
         </is>
       </c>
       <c r="I337" t="inlineStr">

</xml_diff>